<commit_message>
just increased the height of the alert block because it was looking very weird before.
</commit_message>
<xml_diff>
--- a/Attendance Tracker.xlsx
+++ b/Attendance Tracker.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oneibm4\group-project-25-1-the-anti-statics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\para12\Desktop\group-project-25-1-the-anti-statics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{885F4027-F986-4491-9FE9-4C49BF4E6C64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1E4A079-361E-404E-834A-EC7507EB0EFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3570" yWindow="1065" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -509,7 +509,7 @@
         <v>1</v>
       </c>
       <c r="C7" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D7" s="3" t="b">
         <v>1</v>
@@ -562,20 +562,23 @@
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>45733</v>
+      </c>
       <c r="B10" s="3" t="b">
         <v>0</v>
       </c>
       <c r="C10" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D10" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" s="3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>